<commit_message>
2026-Q3 xlsx: populate return_trend from NAV History
Signed-off-by: hmadhani2024@gmail.com
</commit_message>
<xml_diff>
--- a/quarterly-reports/2026-Q3.xlsx
+++ b/quarterly-reports/2026-Q3.xlsx
@@ -461,12 +461,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Charts'!$A$27:$A$26</f>
+              <f>'Charts'!$A$27:$A$43</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Charts'!$C$26:$B$26</f>
+              <f>'Charts'!$B$27:$B$43</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -495,12 +495,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Charts'!$A$27:$A$26</f>
+              <f>'Charts'!$A$27:$A$43</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Charts'!$D$26:$C$26</f>
+              <f>'Charts'!$C$27:$C$43</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -529,12 +529,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Charts'!$A$27:$A$26</f>
+              <f>'Charts'!$A$27:$A$43</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Charts'!$E$26:$D$26</f>
+              <f>'Charts'!$D$27:$D$43</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1993,11 +1993,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
@@ -2138,6 +2138,244 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C27" s="13" t="n"/>
+      <c r="D27" s="18" t="n">
+        <v>766.08</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B28" s="22" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C28" s="22" t="n"/>
+      <c r="D28" s="21" t="n">
+        <v>766.08</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="29" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="n">
+        <v>100031.19</v>
+      </c>
+      <c r="C29" s="13" t="n"/>
+      <c r="D29" s="18" t="n">
+        <v>770.1900000000001</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B30" s="22" t="n">
+        <v>99001.13</v>
+      </c>
+      <c r="C30" s="22" t="n"/>
+      <c r="D30" s="21" t="n">
+        <v>770.1900000000001</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="29" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="n">
+        <v>98412.97</v>
+      </c>
+      <c r="C31" s="13" t="n"/>
+      <c r="D31" s="18" t="n">
+        <v>757.54</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B32" s="22" t="n">
+        <v>98526.03</v>
+      </c>
+      <c r="C32" s="22" t="n"/>
+      <c r="D32" s="21" t="n">
+        <v>764.29</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="29" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="n">
+        <v>98903.82000000001</v>
+      </c>
+      <c r="C33" s="13" t="n"/>
+      <c r="D33" s="18" t="n">
+        <v>760.88</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B34" s="22" t="n">
+        <v>97296.82000000001</v>
+      </c>
+      <c r="C34" s="22" t="n"/>
+      <c r="D34" s="21" t="n">
+        <v>760.88</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="29" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="n">
+        <v>97198</v>
+      </c>
+      <c r="C35" s="13" t="n"/>
+      <c r="D35" s="18" t="n">
+        <v>754.05</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B36" s="22" t="n">
+        <v>97718.10000000001</v>
+      </c>
+      <c r="C36" s="22" t="n"/>
+      <c r="D36" s="21" t="n">
+        <v>762.6</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="29" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="n">
+        <v>98571.78999999999</v>
+      </c>
+      <c r="C37" s="13" t="n"/>
+      <c r="D37" s="18" t="n">
+        <v>767.48</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B38" s="22" t="n">
+        <v>98959.97</v>
+      </c>
+      <c r="C38" s="22" t="n"/>
+      <c r="D38" s="21" t="n">
+        <v>767.48</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="29" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="n">
+        <v>99585.03999999999</v>
+      </c>
+      <c r="C39" s="13" t="n"/>
+      <c r="D39" s="18" t="n">
+        <v>770.71</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B40" s="22" t="n">
+        <v>98790.46000000001</v>
+      </c>
+      <c r="C40" s="22" t="n"/>
+      <c r="D40" s="21" t="n">
+        <v>767.8099999999999</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="29" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="n">
+        <v>98649.27</v>
+      </c>
+      <c r="C41" s="13" t="n"/>
+      <c r="D41" s="18" t="n">
+        <v>767.38</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B42" s="22" t="n">
+        <v>98442.34</v>
+      </c>
+      <c r="C42" s="22" t="n"/>
+      <c r="D42" s="21" t="n">
+        <v>765.63</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="29" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B43" s="13" t="n">
+        <v>98660.21000000001</v>
+      </c>
+      <c r="C43" s="13" t="n"/>
+      <c r="D43" s="18" t="n">
+        <v>765.02</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>